<commit_message>
test(login): add TC_LOGIN_001 login form display
</commit_message>
<xml_diff>
--- a/test_cases/login_test_cases.xlsx
+++ b/test_cases/login_test_cases.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -476,6 +476,31 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Hiển thị đầy đủ giao diện đăng nhập</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>verify_form</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
test(login): add TC_LOGIN_002 password masking
</commit_message>
<xml_diff>
--- a/test_cases/login_test_cases.xlsx
+++ b/test_cases/login_test_cases.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -492,10 +492,36 @@
           <t>verify_form</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Che mật khẩu khi người dùng nhập</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>verify_password_mask</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>MatKhau_Demo_123!</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>

</xml_diff>

<commit_message>
test(login): add TC_LOGIN_003 empty credentials
</commit_message>
<xml_diff>
--- a/test_cases/login_test_cases.xlsx
+++ b/test_cases/login_test_cases.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -514,14 +514,41 @@
           <t>verify_password_mask</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>MatKhau_Demo_123!</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Bỏ trống tên đăng nhập và mật khẩu</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>submit_login</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Bạn chưa nhập tên đăng nhập</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>

</xml_diff>

<commit_message>
test(login): add TC_LOGIN_004 empty username
</commit_message>
<xml_diff>
--- a/test_cases/login_test_cases.xlsx
+++ b/test_cases/login_test_cases.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -541,14 +541,45 @@
           <t>submit_login</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>Bạn chưa nhập tên đăng nhập</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bỏ trống tên đăng nhập</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>submit_login</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>MatKhau_Demo_123!</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Bạn chưa nhập tên đăng nhập</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>

</xml_diff>

<commit_message>
test(login): add TC_LOGIN_005 empty password
</commit_message>
<xml_diff>
--- a/test_cases/login_test_cases.xlsx
+++ b/test_cases/login_test_cases.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -568,7 +568,6 @@
           <t>submit_login</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>MatKhau_Demo_123!</t>
@@ -580,6 +579,39 @@
         </is>
       </c>
       <c r="G5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Bỏ trống mật khẩu</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>submit_login</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>automation_demo_user</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Bạn chưa nhập mật khẩu</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>

</xml_diff>

<commit_message>
test(login): add TC_LOGIN_006 invalid credentials
</commit_message>
<xml_diff>
--- a/test_cases/login_test_cases.xlsx
+++ b/test_cases/login_test_cases.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -605,13 +605,49 @@
           <t>automation_demo_user</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>Bạn chưa nhập mật khẩu</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Đăng nhập với tài khoản không hợp lệ</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>submit_login</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>__selenium_nonexistent_user_6451071052__</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>InvalidPass_123!</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Tài khoản hoặc mật khẩu không đúng.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>

</xml_diff>

<commit_message>
feat: complete login automation suite with Allure report
</commit_message>
<xml_diff>
--- a/test_cases/login_test_cases.xlsx
+++ b/test_cases/login_test_cases.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -653,6 +653,188 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Đăng nhập bằng tài khoản hợp lệ</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>valid_login</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Gửi form đăng nhập bằng phím Enter</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>submit_with_enter</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>__selenium_nonexistent_user_6451071052__</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>InvalidPass_123!</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Tài khoản hoặc mật khẩu không đúng.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Chọn Giữ tôi luôn đăng nhập</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>toggle_remember</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Mở trang quên mật khẩu</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>forgot_password</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>/Login/GetPass</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Chuyển đến đăng nhập e-mail UTC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>utc_sso</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>accounts.google.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Tên đăng nhập có khoảng trắng đầu cuối</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>submit_login</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  __selenium_nonexistent_user_6451071052__  </t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>InvalidPass_123!</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Tài khoản hoặc mật khẩu không đúng.</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>